<commit_message>
feat: super analizador unificado + calculadora de value integrada con rangos dinámicos
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="152">
   <si>
     <t>Jugador / Favorito</t>
   </si>
@@ -101,6 +101,372 @@
   </si>
   <si>
     <t>Kilian Feldbausch</t>
+  </si>
+  <si>
+    <t>Laslo Djere</t>
+  </si>
+  <si>
+    <t>Sorana Cirstea</t>
+  </si>
+  <si>
+    <t>Karen Khachanov</t>
+  </si>
+  <si>
+    <t>Franco Agamenone</t>
+  </si>
+  <si>
+    <t>Lukas Neumayer</t>
+  </si>
+  <si>
+    <t>Casper Ruud</t>
+  </si>
+  <si>
+    <t>Andrey Rublev</t>
+  </si>
+  <si>
+    <t>Martin Krumich</t>
+  </si>
+  <si>
+    <t>Genaro Alberto Olivieri</t>
+  </si>
+  <si>
+    <t>Peyton Stearns</t>
+  </si>
+  <si>
+    <t>Joao Fonseca</t>
+  </si>
+  <si>
+    <t>Pablo Carreño Busta</t>
+  </si>
+  <si>
+    <t>Radu Albot</t>
+  </si>
+  <si>
+    <t>Matteo Berrettini</t>
+  </si>
+  <si>
+    <t>Flavio Cobolli</t>
+  </si>
+  <si>
+    <t>Felix Auger-Aliassime</t>
+  </si>
+  <si>
+    <t>Diana Shnaider</t>
+  </si>
+  <si>
+    <t>Coco Gauff</t>
+  </si>
+  <si>
+    <t>Dusan Obradovic</t>
+  </si>
+  <si>
+    <t>Aristotelis Thanos</t>
+  </si>
+  <si>
+    <t>Viktor Durasovic</t>
+  </si>
+  <si>
+    <t>Laura Samson</t>
+  </si>
+  <si>
+    <t>Carlo Alberto Caniato</t>
+  </si>
+  <si>
+    <t>Marta Kostyuk</t>
+  </si>
+  <si>
+    <t>Oleg Prihodko</t>
+  </si>
+  <si>
+    <t>Anastasia Potapova</t>
+  </si>
+  <si>
+    <t>Alexander Shevchenko</t>
+  </si>
+  <si>
+    <t>Lucia Cortez Llorca</t>
+  </si>
+  <si>
+    <t>Enrico Dalla Valle</t>
+  </si>
+  <si>
+    <t>Valentin Royer</t>
+  </si>
+  <si>
+    <t>Miguel Damas</t>
+  </si>
+  <si>
+    <t>Alice Tubello</t>
+  </si>
+  <si>
+    <t>Dalibor Svrčina</t>
+  </si>
+  <si>
+    <t>Akasha Urhobo</t>
+  </si>
+  <si>
+    <t>Andreea Prisacariu</t>
+  </si>
+  <si>
+    <t>Vitaliy Sachko</t>
+  </si>
+  <si>
+    <t>Rafael Jodar</t>
+  </si>
+  <si>
+    <t>Leyre Romero Gormaz</t>
+  </si>
+  <si>
+    <t>Diego Dedura-Palomero</t>
+  </si>
+  <si>
+    <t>Tyra Caterina Grant</t>
+  </si>
+  <si>
+    <t>Leolia Jeanjean</t>
+  </si>
+  <si>
+    <t>Caijsa Wilda Hennemann</t>
+  </si>
+  <si>
+    <t>Gonzalo Bueno</t>
+  </si>
+  <si>
+    <t>Roberto Carballés Baena</t>
+  </si>
+  <si>
+    <t>Andrea Pellegrino</t>
+  </si>
+  <si>
+    <t>Emilio Nava</t>
+  </si>
+  <si>
+    <t>Tristan Boyer</t>
+  </si>
+  <si>
+    <t>Pablo Llamas Ruiz</t>
+  </si>
+  <si>
+    <t>Darja Semenistaja</t>
+  </si>
+  <si>
+    <t>Vít Kopřiva</t>
+  </si>
+  <si>
+    <t>Tatiana Prozorova</t>
+  </si>
+  <si>
+    <t>Hynek Bartoň</t>
+  </si>
+  <si>
+    <t>Daniel Merida</t>
+  </si>
+  <si>
+    <t>Sebastián Báez</t>
+  </si>
+  <si>
+    <t>Marco Trungelliti</t>
+  </si>
+  <si>
+    <t>Taro Daniel</t>
+  </si>
+  <si>
+    <t>Alexander Zverev</t>
+  </si>
+  <si>
+    <t>Alex Molčan</t>
+  </si>
+  <si>
+    <t>Luca Nardi</t>
+  </si>
+  <si>
+    <t>Mirra Andreeva</t>
+  </si>
+  <si>
+    <t>Nikolas Sanchez Izquierdo</t>
+  </si>
+  <si>
+    <t>Henrique Rocha</t>
+  </si>
+  <si>
+    <t>Iliyan Radulov</t>
+  </si>
+  <si>
+    <t>David Jorda Sanchis</t>
+  </si>
+  <si>
+    <t>Carlos Maria Zarate</t>
+  </si>
+  <si>
+    <t>Andrea Guerrieri</t>
+  </si>
+  <si>
+    <t>Norbert Gombos</t>
+  </si>
+  <si>
+    <t>Federico Cinà</t>
+  </si>
+  <si>
+    <t>Johan Nikles</t>
+  </si>
+  <si>
+    <t>Jonas Forejtek</t>
+  </si>
+  <si>
+    <t>Luca Staeheli</t>
+  </si>
+  <si>
+    <t>Clement Tabur</t>
+  </si>
+  <si>
+    <t>Alvaro Guillen Meza</t>
+  </si>
+  <si>
+    <t>Vilius Gaubas</t>
+  </si>
+  <si>
+    <t>Alejandro Moro Canas</t>
+  </si>
+  <si>
+    <t>Pedro Martinez</t>
+  </si>
+  <si>
+    <t>Santiago de la Fuente</t>
+  </si>
+  <si>
+    <t>Martina Trevisan</t>
+  </si>
+  <si>
+    <t>Lukas Pokorny</t>
+  </si>
+  <si>
+    <t>Petr Brunclik</t>
+  </si>
+  <si>
+    <t>Joao Lucas Reis da Silva</t>
+  </si>
+  <si>
+    <t>Juan Bautista Torres</t>
+  </si>
+  <si>
+    <t>Zsombor Piros</t>
+  </si>
+  <si>
+    <t>Nuria Brancaccio</t>
+  </si>
+  <si>
+    <t>Alejo Sanchez Quilez</t>
+  </si>
+  <si>
+    <t>Ryan Seggerman</t>
+  </si>
+  <si>
+    <t>Lorenzo Bocchi</t>
+  </si>
+  <si>
+    <t>Miguel Tobon</t>
+  </si>
+  <si>
+    <t>Denis Yevseyev</t>
+  </si>
+  <si>
+    <t>Michael Vrbensky</t>
+  </si>
+  <si>
+    <t>Giorgia Pedone</t>
+  </si>
+  <si>
+    <t>Matteo Martineau</t>
+  </si>
+  <si>
+    <t>Deborah Chiesa</t>
+  </si>
+  <si>
+    <t>Franco Ribero</t>
+  </si>
+  <si>
+    <t>Sebastian Ofner</t>
+  </si>
+  <si>
+    <t>Cosme Rolland de Ravel</t>
+  </si>
+  <si>
+    <t>Svyatoslav Gulin</t>
+  </si>
+  <si>
+    <t>Damir Dzumhur</t>
+  </si>
+  <si>
+    <t>Guido Ivan Justo</t>
+  </si>
+  <si>
+    <t>Jacopo Vasami</t>
+  </si>
+  <si>
+    <t>Max Alcala Gurri</t>
+  </si>
+  <si>
+    <t>Gilles-Arnaud Bailly</t>
+  </si>
+  <si>
+    <t>Julia Grabher</t>
+  </si>
+  <si>
+    <t>Jan Choinski</t>
+  </si>
+  <si>
+    <t>Manas Dhamne</t>
+  </si>
+  <si>
+    <t>Ane Mintegi del Olmo</t>
+  </si>
+  <si>
+    <t>Fiona Ferro</t>
+  </si>
+  <si>
+    <t>Robin Bertrand</t>
+  </si>
+  <si>
+    <t>Eliakim Coulibaly</t>
+  </si>
+  <si>
+    <t>Michiel de Krom</t>
+  </si>
+  <si>
+    <t>Pedro Sakamoto</t>
+  </si>
+  <si>
+    <t>Pietro Orlando Fellin</t>
+  </si>
+  <si>
+    <t>Rares Teodor Pieleanu</t>
+  </si>
+  <si>
+    <t>Miriam Bulgaru</t>
+  </si>
+  <si>
+    <t>Mayar Sherif</t>
+  </si>
+  <si>
+    <t>Carlos Sanchez Jover</t>
+  </si>
+  <si>
+    <t>Ekaterine Gorgodze</t>
+  </si>
+  <si>
+    <t>Peter Fajta</t>
+  </si>
+  <si>
+    <t>Mili Poljicak</t>
+  </si>
+  <si>
+    <t>Andrej Nedic</t>
+  </si>
+  <si>
+    <t>Dominic Stricker</t>
+  </si>
+  <si>
+    <t>Tanguy Genier</t>
   </si>
 </sst>
 </file>
@@ -969,6 +1335,18 @@
       <c r="J27" s="4"/>
     </row>
     <row r="28">
+      <c r="A28" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1.83</v>
+      </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -977,6 +1355,18 @@
       <c r="J28" s="4"/>
     </row>
     <row r="29">
+      <c r="A29" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="8">
+        <v>1.8</v>
+      </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -985,6 +1375,18 @@
       <c r="J29" s="4"/>
     </row>
     <row r="30">
+      <c r="A30" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="8">
+        <v>1.28</v>
+      </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -993,6 +1395,18 @@
       <c r="J30" s="4"/>
     </row>
     <row r="31">
+      <c r="A31" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="8">
+        <v>1.36</v>
+      </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -1001,6 +1415,18 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32">
+      <c r="A32" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="8">
+        <v>1.3</v>
+      </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -1009,6 +1435,18 @@
       <c r="J32" s="4"/>
     </row>
     <row r="33">
+      <c r="A33" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="8">
+        <v>1.28</v>
+      </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -1017,6 +1455,18 @@
       <c r="J33" s="4"/>
     </row>
     <row r="34">
+      <c r="A34" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -1025,6 +1475,18 @@
       <c r="J34" s="4"/>
     </row>
     <row r="35">
+      <c r="A35" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -1033,6 +1495,18 @@
       <c r="J35" s="4"/>
     </row>
     <row r="36">
+      <c r="A36" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="8">
+        <v>1.36</v>
+      </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -1041,6 +1515,18 @@
       <c r="J36" s="4"/>
     </row>
     <row r="37">
+      <c r="A37" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="8">
+        <v>2.75</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -1049,6 +1535,18 @@
       <c r="J37" s="4"/>
     </row>
     <row r="38">
+      <c r="A38" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="8">
+        <v>3.4</v>
+      </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -1057,6 +1555,18 @@
       <c r="J38" s="4"/>
     </row>
     <row r="39">
+      <c r="A39" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="8">
+        <v>2.75</v>
+      </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -1065,6 +1575,18 @@
       <c r="J39" s="4"/>
     </row>
     <row r="40">
+      <c r="A40" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" s="8">
+        <v>3.0</v>
+      </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -1073,6 +1595,18 @@
       <c r="J40" s="4"/>
     </row>
     <row r="41">
+      <c r="A41" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="8">
+        <v>3.0</v>
+      </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -1081,6 +1615,18 @@
       <c r="J41" s="4"/>
     </row>
     <row r="42">
+      <c r="A42" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="6">
+        <v>0.61</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -1089,6 +1635,18 @@
       <c r="J42" s="4"/>
     </row>
     <row r="43">
+      <c r="A43" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D43" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -1097,6 +1655,18 @@
       <c r="J43" s="4"/>
     </row>
     <row r="44">
+      <c r="A44" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D44" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -1105,6 +1675,18 @@
       <c r="J44" s="4"/>
     </row>
     <row r="45">
+      <c r="A45" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -1113,6 +1695,18 @@
       <c r="J45" s="4"/>
     </row>
     <row r="46">
+      <c r="A46" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="8">
+        <v>1.28</v>
+      </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -1121,6 +1715,18 @@
       <c r="J46" s="4"/>
     </row>
     <row r="47">
+      <c r="A47" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="8">
+        <v>2.75</v>
+      </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -1129,6 +1735,18 @@
       <c r="J47" s="4"/>
     </row>
     <row r="48">
+      <c r="A48" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" s="6">
+        <v>0.66</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D48" s="8">
+        <v>1.36</v>
+      </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
@@ -1137,6 +1755,18 @@
       <c r="J48" s="4"/>
     </row>
     <row r="49">
+      <c r="A49" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="6">
+        <v>0.73</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -1145,6 +1775,18 @@
       <c r="J49" s="4"/>
     </row>
     <row r="50">
+      <c r="A50" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="8">
+        <v>1.3</v>
+      </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -1153,6 +1795,18 @@
       <c r="J50" s="4"/>
     </row>
     <row r="51">
+      <c r="A51" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" s="6">
+        <v>0.67</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="8">
+        <v>2.62</v>
+      </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -1161,6 +1815,18 @@
       <c r="J51" s="4"/>
     </row>
     <row r="52">
+      <c r="A52" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -1169,6 +1835,18 @@
       <c r="J52" s="4"/>
     </row>
     <row r="53">
+      <c r="A53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D53" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -1177,6 +1855,18 @@
       <c r="J53" s="4"/>
     </row>
     <row r="54">
+      <c r="A54" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D54" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -1185,6 +1875,18 @@
       <c r="J54" s="4"/>
     </row>
     <row r="55">
+      <c r="A55" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B55" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D55" s="8">
+        <v>3.2</v>
+      </c>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -1193,6 +1895,18 @@
       <c r="J55" s="4"/>
     </row>
     <row r="56">
+      <c r="A56" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56" s="8">
+        <v>1.3</v>
+      </c>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -1201,6 +1915,18 @@
       <c r="J56" s="4"/>
     </row>
     <row r="57">
+      <c r="A57" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" s="6">
+        <v>0.73</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -1209,6 +1935,18 @@
       <c r="J57" s="4"/>
     </row>
     <row r="58">
+      <c r="A58" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B58" s="6">
+        <v>0.61</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" s="8">
+        <v>1.3</v>
+      </c>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -1217,6 +1955,18 @@
       <c r="J58" s="4"/>
     </row>
     <row r="59">
+      <c r="A59" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B59" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -1225,6 +1975,18 @@
       <c r="J59" s="4"/>
     </row>
     <row r="60">
+      <c r="A60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" s="8">
+        <v>1.25</v>
+      </c>
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
@@ -1233,6 +1995,18 @@
       <c r="J60" s="4"/>
     </row>
     <row r="61">
+      <c r="A61" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B61" s="6">
+        <v>0.56</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" s="8">
+        <v>3.0</v>
+      </c>
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
@@ -1241,6 +2015,18 @@
       <c r="J61" s="4"/>
     </row>
     <row r="62">
+      <c r="A62" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="8">
+        <v>1.28</v>
+      </c>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
@@ -1249,6 +2035,18 @@
       <c r="J62" s="4"/>
     </row>
     <row r="63">
+      <c r="A63" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D63" s="8">
+        <v>3.5</v>
+      </c>
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
@@ -1257,6 +2055,18 @@
       <c r="J63" s="4"/>
     </row>
     <row r="64">
+      <c r="A64" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" s="6">
+        <v>0.52</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E64" s="4"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
@@ -1265,6 +2075,18 @@
       <c r="J64" s="4"/>
     </row>
     <row r="65">
+      <c r="A65" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B65" s="6">
+        <v>0.74</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" s="8">
+        <v>1.25</v>
+      </c>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -1273,6 +2095,18 @@
       <c r="J65" s="4"/>
     </row>
     <row r="66">
+      <c r="A66" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D66" s="8">
+        <v>1.25</v>
+      </c>
       <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
@@ -1281,6 +2115,18 @@
       <c r="J66" s="4"/>
     </row>
     <row r="67">
+      <c r="A67" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B67" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
@@ -1289,6 +2135,18 @@
       <c r="J67" s="4"/>
     </row>
     <row r="68">
+      <c r="A68" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" s="6">
+        <v>0.51</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D68" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
@@ -1297,6 +2155,18 @@
       <c r="J68" s="4"/>
     </row>
     <row r="69">
+      <c r="A69" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B69" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D69" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
@@ -1305,6 +2175,18 @@
       <c r="J69" s="4"/>
     </row>
     <row r="70">
+      <c r="A70" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B70" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D70" s="8">
+        <v>3.5</v>
+      </c>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
@@ -1313,6 +2195,18 @@
       <c r="J70" s="4"/>
     </row>
     <row r="71">
+      <c r="A71" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B71" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E71" s="4"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
@@ -1321,6 +2215,18 @@
       <c r="J71" s="4"/>
     </row>
     <row r="72">
+      <c r="A72" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B72" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" s="8">
+        <v>1.28</v>
+      </c>
       <c r="E72" s="4"/>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
@@ -1329,6 +2235,18 @@
       <c r="J72" s="4"/>
     </row>
     <row r="73">
+      <c r="A73" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B73" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
@@ -1337,6 +2255,18 @@
       <c r="J73" s="4"/>
     </row>
     <row r="74">
+      <c r="A74" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B74" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D74" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E74" s="4"/>
       <c r="F74" s="4"/>
       <c r="G74" s="4"/>
@@ -1345,6 +2275,18 @@
       <c r="J74" s="4"/>
     </row>
     <row r="75">
+      <c r="A75" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" s="8">
+        <v>1.36</v>
+      </c>
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
       <c r="G75" s="4"/>
@@ -1353,6 +2295,18 @@
       <c r="J75" s="4"/>
     </row>
     <row r="76">
+      <c r="A76" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B76" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D76" s="8">
+        <v>3.0</v>
+      </c>
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
@@ -1361,6 +2315,18 @@
       <c r="J76" s="4"/>
     </row>
     <row r="77">
+      <c r="A77" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B77" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D77" s="8">
+        <v>1.33</v>
+      </c>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
@@ -1369,6 +2335,18 @@
       <c r="J77" s="4"/>
     </row>
     <row r="78">
+      <c r="A78" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B78" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D78" s="8">
+        <v>1.4</v>
+      </c>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
@@ -1377,6 +2355,18 @@
       <c r="J78" s="4"/>
     </row>
     <row r="79">
+      <c r="A79" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B79" s="6">
+        <v>0.74</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D79" s="8">
+        <v>1.44</v>
+      </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
       <c r="G79" s="4"/>
@@ -1385,6 +2375,18 @@
       <c r="J79" s="4"/>
     </row>
     <row r="80">
+      <c r="A80" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B80" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" s="8">
+        <v>1.22</v>
+      </c>
       <c r="E80" s="4"/>
       <c r="F80" s="4"/>
       <c r="G80" s="4"/>
@@ -1392,6 +2394,2306 @@
       <c r="I80" s="4"/>
       <c r="J80" s="4"/>
     </row>
+    <row r="81">
+      <c r="A81" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B81" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D81" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="4"/>
+      <c r="H81" s="4"/>
+      <c r="I81" s="4"/>
+      <c r="J81" s="4"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B82" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E82" s="4"/>
+      <c r="F82" s="4"/>
+      <c r="G82" s="4"/>
+      <c r="H82" s="4"/>
+      <c r="I82" s="4"/>
+      <c r="J82" s="4"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B83" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D83" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="4"/>
+      <c r="H83" s="4"/>
+      <c r="I83" s="4"/>
+      <c r="J83" s="4"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B84" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D84" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E84" s="4"/>
+      <c r="F84" s="4"/>
+      <c r="G84" s="4"/>
+      <c r="H84" s="4"/>
+      <c r="I84" s="4"/>
+      <c r="J84" s="4"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B85" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D85" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E85" s="4"/>
+      <c r="F85" s="4"/>
+      <c r="G85" s="4"/>
+      <c r="H85" s="4"/>
+      <c r="I85" s="4"/>
+      <c r="J85" s="4"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B86" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+      <c r="G86" s="4"/>
+      <c r="H86" s="4"/>
+      <c r="I86" s="4"/>
+      <c r="J86" s="4"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B87" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C87" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+      <c r="G87" s="4"/>
+      <c r="H87" s="4"/>
+      <c r="I87" s="4"/>
+      <c r="J87" s="4"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B88" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D88" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E88" s="4"/>
+      <c r="F88" s="4"/>
+      <c r="G88" s="4"/>
+      <c r="H88" s="4"/>
+      <c r="I88" s="4"/>
+      <c r="J88" s="4"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B89" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D89" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E89" s="4"/>
+      <c r="F89" s="4"/>
+      <c r="G89" s="4"/>
+      <c r="H89" s="4"/>
+      <c r="I89" s="4"/>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B90" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D90" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E90" s="4"/>
+      <c r="F90" s="4"/>
+      <c r="G90" s="4"/>
+      <c r="H90" s="4"/>
+      <c r="I90" s="4"/>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B91" s="6">
+        <v>0.81</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
+      <c r="G91" s="4"/>
+      <c r="H91" s="4"/>
+      <c r="I91" s="4"/>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B92" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D92" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E92" s="4"/>
+      <c r="F92" s="4"/>
+      <c r="G92" s="4"/>
+      <c r="H92" s="4"/>
+      <c r="I92" s="4"/>
+      <c r="J92" s="4"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B93" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D93" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+      <c r="G93" s="4"/>
+      <c r="H93" s="4"/>
+      <c r="I93" s="4"/>
+      <c r="J93" s="4"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B94" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E94" s="4"/>
+      <c r="F94" s="4"/>
+      <c r="G94" s="4"/>
+      <c r="H94" s="4"/>
+      <c r="I94" s="4"/>
+      <c r="J94" s="4"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B95" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D95" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="4"/>
+      <c r="H95" s="4"/>
+      <c r="I95" s="4"/>
+      <c r="J95" s="4"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B96" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D96" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E96" s="4"/>
+      <c r="F96" s="4"/>
+      <c r="G96" s="4"/>
+      <c r="H96" s="4"/>
+      <c r="I96" s="4"/>
+      <c r="J96" s="4"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B97" s="6">
+        <v>0.66</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D97" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="E97" s="4"/>
+      <c r="F97" s="4"/>
+      <c r="G97" s="4"/>
+      <c r="H97" s="4"/>
+      <c r="I97" s="4"/>
+      <c r="J97" s="4"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B98" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+      <c r="H98" s="4"/>
+      <c r="I98" s="4"/>
+      <c r="J98" s="4"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B99" s="6">
+        <v>0.69</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D99" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="4"/>
+      <c r="H99" s="4"/>
+      <c r="I99" s="4"/>
+      <c r="J99" s="4"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B100" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D100" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="4"/>
+      <c r="J100" s="4"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B101" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C101" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D101" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E101" s="4"/>
+      <c r="F101" s="4"/>
+      <c r="G101" s="4"/>
+      <c r="H101" s="4"/>
+      <c r="I101" s="4"/>
+      <c r="J101" s="4"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B102" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D102" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E102" s="4"/>
+      <c r="F102" s="4"/>
+      <c r="G102" s="4"/>
+      <c r="H102" s="4"/>
+      <c r="I102" s="4"/>
+      <c r="J102" s="4"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B103" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D103" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="4"/>
+      <c r="H103" s="4"/>
+      <c r="I103" s="4"/>
+      <c r="J103" s="4"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B104" s="6">
+        <v>0.81</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D104" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
+      <c r="G104" s="4"/>
+      <c r="H104" s="4"/>
+      <c r="I104" s="4"/>
+      <c r="J104" s="4"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B105" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D105" s="8">
+        <v>3.75</v>
+      </c>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="4"/>
+      <c r="H105" s="4"/>
+      <c r="I105" s="4"/>
+      <c r="J105" s="4"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B106" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C106" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D106" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E106" s="4"/>
+      <c r="F106" s="4"/>
+      <c r="G106" s="4"/>
+      <c r="H106" s="4"/>
+      <c r="I106" s="4"/>
+      <c r="J106" s="4"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B107" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D107" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="4"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B108" s="6">
+        <v>0.56</v>
+      </c>
+      <c r="C108" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D108" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E108" s="4"/>
+      <c r="F108" s="4"/>
+      <c r="G108" s="4"/>
+      <c r="H108" s="4"/>
+      <c r="I108" s="4"/>
+      <c r="J108" s="4"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B109" s="6">
+        <v>0.81</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D109" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E109" s="4"/>
+      <c r="F109" s="4"/>
+      <c r="G109" s="4"/>
+      <c r="H109" s="4"/>
+      <c r="I109" s="4"/>
+      <c r="J109" s="4"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B110" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D110" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E110" s="4"/>
+      <c r="F110" s="4"/>
+      <c r="G110" s="4"/>
+      <c r="H110" s="4"/>
+      <c r="I110" s="4"/>
+      <c r="J110" s="4"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B111" s="6">
+        <v>0.59</v>
+      </c>
+      <c r="C111" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D111" s="8">
+        <v>3.75</v>
+      </c>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="4"/>
+      <c r="H111" s="4"/>
+      <c r="I111" s="4"/>
+      <c r="J111" s="4"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B112" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D112" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E112" s="4"/>
+      <c r="F112" s="4"/>
+      <c r="G112" s="4"/>
+      <c r="H112" s="4"/>
+      <c r="I112" s="4"/>
+      <c r="J112" s="4"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" s="6">
+        <v>0.84</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D113" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="E113" s="4"/>
+      <c r="F113" s="4"/>
+      <c r="G113" s="4"/>
+      <c r="H113" s="4"/>
+      <c r="I113" s="4"/>
+      <c r="J113" s="4"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B114" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D114" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="E114" s="4"/>
+      <c r="F114" s="4"/>
+      <c r="G114" s="4"/>
+      <c r="H114" s="4"/>
+      <c r="I114" s="4"/>
+      <c r="J114" s="4"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B115" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D115" s="8">
+        <v>3.75</v>
+      </c>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="4"/>
+      <c r="H115" s="4"/>
+      <c r="I115" s="4"/>
+      <c r="J115" s="4"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B116" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D116" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E116" s="4"/>
+      <c r="F116" s="4"/>
+      <c r="G116" s="4"/>
+      <c r="H116" s="4"/>
+      <c r="I116" s="4"/>
+      <c r="J116" s="4"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B117" s="6">
+        <v>0.61</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D117" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E117" s="4"/>
+      <c r="F117" s="4"/>
+      <c r="G117" s="4"/>
+      <c r="H117" s="4"/>
+      <c r="I117" s="4"/>
+      <c r="J117" s="4"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B118" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D118" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E118" s="4"/>
+      <c r="F118" s="4"/>
+      <c r="G118" s="4"/>
+      <c r="H118" s="4"/>
+      <c r="I118" s="4"/>
+      <c r="J118" s="4"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B119" s="6">
+        <v>0.69</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D119" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E119" s="4"/>
+      <c r="F119" s="4"/>
+      <c r="G119" s="4"/>
+      <c r="H119" s="4"/>
+      <c r="I119" s="4"/>
+      <c r="J119" s="4"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B120" s="6">
+        <v>0.66</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D120" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E120" s="4"/>
+      <c r="F120" s="4"/>
+      <c r="G120" s="4"/>
+      <c r="H120" s="4"/>
+      <c r="I120" s="4"/>
+      <c r="J120" s="4"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B121" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D121" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E121" s="4"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="4"/>
+      <c r="H121" s="4"/>
+      <c r="I121" s="4"/>
+      <c r="J121" s="4"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B122" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D122" s="8">
+        <v>1.22</v>
+      </c>
+      <c r="E122" s="4"/>
+      <c r="F122" s="4"/>
+      <c r="G122" s="4"/>
+      <c r="H122" s="4"/>
+      <c r="I122" s="4"/>
+      <c r="J122" s="4"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B123" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D123" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+      <c r="H123" s="4"/>
+      <c r="I123" s="4"/>
+      <c r="J123" s="4"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B124" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D124" s="8">
+        <v>3.75</v>
+      </c>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4"/>
+      <c r="G124" s="4"/>
+      <c r="H124" s="4"/>
+      <c r="I124" s="4"/>
+      <c r="J124" s="4"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B125" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D125" s="8">
+        <v>2.62</v>
+      </c>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4"/>
+      <c r="G125" s="4"/>
+      <c r="H125" s="4"/>
+      <c r="I125" s="4"/>
+      <c r="J125" s="4"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B126" s="6">
+        <v>0.66</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D126" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E126" s="4"/>
+      <c r="F126" s="4"/>
+      <c r="G126" s="4"/>
+      <c r="H126" s="4"/>
+      <c r="I126" s="4"/>
+      <c r="J126" s="4"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B127" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C127" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D127" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E127" s="4"/>
+      <c r="F127" s="4"/>
+      <c r="G127" s="4"/>
+      <c r="H127" s="4"/>
+      <c r="I127" s="4"/>
+      <c r="J127" s="4"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B128" s="6">
+        <v>0.56</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D128" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4"/>
+      <c r="G128" s="4"/>
+      <c r="H128" s="4"/>
+      <c r="I128" s="4"/>
+      <c r="J128" s="4"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B129" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D129" s="8">
+        <v>1.22</v>
+      </c>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="4"/>
+      <c r="H129" s="4"/>
+      <c r="I129" s="4"/>
+      <c r="J129" s="4"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B130" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D130" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E130" s="4"/>
+      <c r="F130" s="4"/>
+      <c r="G130" s="4"/>
+      <c r="H130" s="4"/>
+      <c r="I130" s="4"/>
+      <c r="J130" s="4"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B131" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D131" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="4"/>
+      <c r="H131" s="4"/>
+      <c r="I131" s="4"/>
+      <c r="J131" s="4"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B132" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C132" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D132" s="8">
+        <v>1.22</v>
+      </c>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4"/>
+      <c r="G132" s="4"/>
+      <c r="H132" s="4"/>
+      <c r="I132" s="4"/>
+      <c r="J132" s="4"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B133" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D133" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="4"/>
+      <c r="H133" s="4"/>
+      <c r="I133" s="4"/>
+      <c r="J133" s="4"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B134" s="6">
+        <v>0.63</v>
+      </c>
+      <c r="C134" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D134" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E134" s="4"/>
+      <c r="F134" s="4"/>
+      <c r="G134" s="4"/>
+      <c r="H134" s="4"/>
+      <c r="I134" s="4"/>
+      <c r="J134" s="4"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B135" s="6">
+        <v>0.57</v>
+      </c>
+      <c r="C135" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D135" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+      <c r="G135" s="4"/>
+      <c r="H135" s="4"/>
+      <c r="I135" s="4"/>
+      <c r="J135" s="4"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B136" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C136" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D136" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E136" s="4"/>
+      <c r="F136" s="4"/>
+      <c r="G136" s="4"/>
+      <c r="H136" s="4"/>
+      <c r="I136" s="4"/>
+      <c r="J136" s="4"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B137" s="6">
+        <v>0.57</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D137" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E137" s="4"/>
+      <c r="F137" s="4"/>
+      <c r="G137" s="4"/>
+      <c r="H137" s="4"/>
+      <c r="I137" s="4"/>
+      <c r="J137" s="4"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B138" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C138" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D138" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E138" s="4"/>
+      <c r="F138" s="4"/>
+      <c r="G138" s="4"/>
+      <c r="H138" s="4"/>
+      <c r="I138" s="4"/>
+      <c r="J138" s="4"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B139" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C139" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D139" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="4"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B140" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C140" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D140" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E140" s="4"/>
+      <c r="F140" s="4"/>
+      <c r="G140" s="4"/>
+      <c r="H140" s="4"/>
+      <c r="I140" s="4"/>
+      <c r="J140" s="4"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B141" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C141" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D141" s="8">
+        <v>2.62</v>
+      </c>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+      <c r="H141" s="4"/>
+      <c r="I141" s="4"/>
+      <c r="J141" s="4"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B142" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C142" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D142" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="E142" s="4"/>
+      <c r="F142" s="4"/>
+      <c r="G142" s="4"/>
+      <c r="H142" s="4"/>
+      <c r="I142" s="4"/>
+      <c r="J142" s="4"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B143" s="6">
+        <v>0.77</v>
+      </c>
+      <c r="C143" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D143" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="4"/>
+      <c r="H143" s="4"/>
+      <c r="I143" s="4"/>
+      <c r="J143" s="4"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B144" s="6">
+        <v>0.84</v>
+      </c>
+      <c r="C144" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D144" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="E144" s="4"/>
+      <c r="F144" s="4"/>
+      <c r="G144" s="4"/>
+      <c r="H144" s="4"/>
+      <c r="I144" s="4"/>
+      <c r="J144" s="4"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B145" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C145" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D145" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="4"/>
+      <c r="H145" s="4"/>
+      <c r="I145" s="4"/>
+      <c r="J145" s="4"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B146" s="6">
+        <v>0.73</v>
+      </c>
+      <c r="C146" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D146" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E146" s="4"/>
+      <c r="F146" s="4"/>
+      <c r="G146" s="4"/>
+      <c r="H146" s="4"/>
+      <c r="I146" s="4"/>
+      <c r="J146" s="4"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B147" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C147" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D147" s="8">
+        <v>2.62</v>
+      </c>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="4"/>
+      <c r="H147" s="4"/>
+      <c r="I147" s="4"/>
+      <c r="J147" s="4"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B148" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D148" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E148" s="4"/>
+      <c r="F148" s="4"/>
+      <c r="G148" s="4"/>
+      <c r="H148" s="4"/>
+      <c r="I148" s="4"/>
+      <c r="J148" s="4"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B149" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C149" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D149" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="4"/>
+      <c r="H149" s="4"/>
+      <c r="I149" s="4"/>
+      <c r="J149" s="4"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B150" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C150" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D150" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E150" s="4"/>
+      <c r="F150" s="4"/>
+      <c r="G150" s="4"/>
+      <c r="H150" s="4"/>
+      <c r="I150" s="4"/>
+      <c r="J150" s="4"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B151" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C151" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D151" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="4"/>
+      <c r="H151" s="4"/>
+      <c r="I151" s="4"/>
+      <c r="J151" s="4"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B152" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C152" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D152" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E152" s="4"/>
+      <c r="F152" s="4"/>
+      <c r="G152" s="4"/>
+      <c r="H152" s="4"/>
+      <c r="I152" s="4"/>
+      <c r="J152" s="4"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B153" s="6">
+        <v>0.74</v>
+      </c>
+      <c r="C153" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D153" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="4"/>
+      <c r="H153" s="4"/>
+      <c r="I153" s="4"/>
+      <c r="J153" s="4"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B154" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D154" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+      <c r="G154" s="4"/>
+      <c r="H154" s="4"/>
+      <c r="I154" s="4"/>
+      <c r="J154" s="4"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B155" s="6">
+        <v>0.77</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D155" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="4"/>
+      <c r="H155" s="4"/>
+      <c r="I155" s="4"/>
+      <c r="J155" s="4"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B156" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C156" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D156" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E156" s="4"/>
+      <c r="F156" s="4"/>
+      <c r="G156" s="4"/>
+      <c r="H156" s="4"/>
+      <c r="I156" s="4"/>
+      <c r="J156" s="4"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B157" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C157" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D157" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="4"/>
+      <c r="H157" s="4"/>
+      <c r="I157" s="4"/>
+      <c r="J157" s="4"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B158" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C158" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D158" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E158" s="4"/>
+      <c r="F158" s="4"/>
+      <c r="G158" s="4"/>
+      <c r="H158" s="4"/>
+      <c r="I158" s="4"/>
+      <c r="J158" s="4"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B159" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C159" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D159" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="4"/>
+      <c r="H159" s="4"/>
+      <c r="I159" s="4"/>
+      <c r="J159" s="4"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B160" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C160" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D160" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E160" s="4"/>
+      <c r="F160" s="4"/>
+      <c r="G160" s="4"/>
+      <c r="H160" s="4"/>
+      <c r="I160" s="4"/>
+      <c r="J160" s="4"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B161" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C161" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D161" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="4"/>
+      <c r="H161" s="4"/>
+      <c r="I161" s="4"/>
+      <c r="J161" s="4"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B162" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D162" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E162" s="4"/>
+      <c r="F162" s="4"/>
+      <c r="G162" s="4"/>
+      <c r="H162" s="4"/>
+      <c r="I162" s="4"/>
+      <c r="J162" s="4"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B163" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C163" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D163" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="4"/>
+      <c r="H163" s="4"/>
+      <c r="I163" s="4"/>
+      <c r="J163" s="4"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B164" s="6">
+        <v>0.69</v>
+      </c>
+      <c r="C164" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D164" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E164" s="4"/>
+      <c r="F164" s="4"/>
+      <c r="G164" s="4"/>
+      <c r="H164" s="4"/>
+      <c r="I164" s="4"/>
+      <c r="J164" s="4"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B165" s="6">
+        <v>0.66</v>
+      </c>
+      <c r="C165" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D165" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="4"/>
+      <c r="H165" s="4"/>
+      <c r="I165" s="4"/>
+      <c r="J165" s="4"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B166" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="C166" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D166" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E166" s="4"/>
+      <c r="F166" s="4"/>
+      <c r="G166" s="4"/>
+      <c r="H166" s="4"/>
+      <c r="I166" s="4"/>
+      <c r="J166" s="4"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B167" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C167" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D167" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E167" s="4"/>
+      <c r="F167" s="4"/>
+      <c r="G167" s="4"/>
+      <c r="H167" s="4"/>
+      <c r="I167" s="4"/>
+      <c r="J167" s="4"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B168" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C168" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D168" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E168" s="4"/>
+      <c r="F168" s="4"/>
+      <c r="G168" s="4"/>
+      <c r="H168" s="4"/>
+      <c r="I168" s="4"/>
+      <c r="J168" s="4"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B169" s="6">
+        <v>0.67</v>
+      </c>
+      <c r="C169" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D169" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="4"/>
+      <c r="H169" s="4"/>
+      <c r="I169" s="4"/>
+      <c r="J169" s="4"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B170" s="6">
+        <v>0.74</v>
+      </c>
+      <c r="C170" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D170" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E170" s="4"/>
+      <c r="F170" s="4"/>
+      <c r="G170" s="4"/>
+      <c r="H170" s="4"/>
+      <c r="I170" s="4"/>
+      <c r="J170" s="4"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B171" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C171" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D171" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E171" s="4"/>
+      <c r="F171" s="4"/>
+      <c r="G171" s="4"/>
+      <c r="H171" s="4"/>
+      <c r="I171" s="4"/>
+      <c r="J171" s="4"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B172" s="6">
+        <v>0.79</v>
+      </c>
+      <c r="C172" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D172" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E172" s="4"/>
+      <c r="F172" s="4"/>
+      <c r="G172" s="4"/>
+      <c r="H172" s="4"/>
+      <c r="I172" s="4"/>
+      <c r="J172" s="4"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B173" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C173" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D173" s="8">
+        <v>3.0</v>
+      </c>
+      <c r="E173" s="4"/>
+      <c r="F173" s="4"/>
+      <c r="G173" s="4"/>
+      <c r="H173" s="4"/>
+      <c r="I173" s="4"/>
+      <c r="J173" s="4"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B174" s="6">
+        <v>0.73</v>
+      </c>
+      <c r="C174" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D174" s="8">
+        <v>3.75</v>
+      </c>
+      <c r="E174" s="4"/>
+      <c r="F174" s="4"/>
+      <c r="G174" s="4"/>
+      <c r="H174" s="4"/>
+      <c r="I174" s="4"/>
+      <c r="J174" s="4"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B175" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="C175" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D175" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E175" s="4"/>
+      <c r="F175" s="4"/>
+      <c r="G175" s="4"/>
+      <c r="H175" s="4"/>
+      <c r="I175" s="4"/>
+      <c r="J175" s="4"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B176" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C176" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D176" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E176" s="4"/>
+      <c r="F176" s="4"/>
+      <c r="G176" s="4"/>
+      <c r="H176" s="4"/>
+      <c r="I176" s="4"/>
+      <c r="J176" s="4"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B177" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C177" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D177" s="8">
+        <v>1.25</v>
+      </c>
+      <c r="E177" s="4"/>
+      <c r="F177" s="4"/>
+      <c r="G177" s="4"/>
+      <c r="H177" s="4"/>
+      <c r="I177" s="4"/>
+      <c r="J177" s="4"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B178" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C178" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D178" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E178" s="4"/>
+      <c r="F178" s="4"/>
+      <c r="G178" s="4"/>
+      <c r="H178" s="4"/>
+      <c r="I178" s="4"/>
+      <c r="J178" s="4"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B179" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C179" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D179" s="8">
+        <v>1.36</v>
+      </c>
+      <c r="E179" s="4"/>
+      <c r="F179" s="4"/>
+      <c r="G179" s="4"/>
+      <c r="H179" s="4"/>
+      <c r="I179" s="4"/>
+      <c r="J179" s="4"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B180" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C180" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D180" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="E180" s="4"/>
+      <c r="F180" s="4"/>
+      <c r="G180" s="4"/>
+      <c r="H180" s="4"/>
+      <c r="I180" s="4"/>
+      <c r="J180" s="4"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B181" s="6">
+        <v>0.53</v>
+      </c>
+      <c r="C181" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D181" s="8">
+        <v>3.0</v>
+      </c>
+      <c r="E181" s="4"/>
+      <c r="F181" s="4"/>
+      <c r="G181" s="4"/>
+      <c r="H181" s="4"/>
+      <c r="I181" s="4"/>
+      <c r="J181" s="4"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B182" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="C182" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D182" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E182" s="4"/>
+      <c r="F182" s="4"/>
+      <c r="G182" s="4"/>
+      <c r="H182" s="4"/>
+      <c r="I182" s="4"/>
+      <c r="J182" s="4"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B183" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="C183" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D183" s="8">
+        <v>3.0</v>
+      </c>
+      <c r="E183" s="4"/>
+      <c r="F183" s="4"/>
+      <c r="G183" s="4"/>
+      <c r="H183" s="4"/>
+      <c r="I183" s="4"/>
+      <c r="J183" s="4"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B184" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C184" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D184" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="4"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B185" s="6">
+        <v>0.73</v>
+      </c>
+      <c r="C185" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D185" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+      <c r="G185" s="4"/>
+      <c r="H185" s="4"/>
+      <c r="I185" s="4"/>
+      <c r="J185" s="4"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B186" s="6">
+        <v>0.88</v>
+      </c>
+      <c r="C186" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D186" s="8">
+        <v>1.28</v>
+      </c>
+      <c r="E186" s="4"/>
+      <c r="F186" s="4"/>
+      <c r="G186" s="4"/>
+      <c r="H186" s="4"/>
+      <c r="I186" s="4"/>
+      <c r="J186" s="4"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B187" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="C187" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D187" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E187" s="4"/>
+      <c r="F187" s="4"/>
+      <c r="G187" s="4"/>
+      <c r="H187" s="4"/>
+      <c r="I187" s="4"/>
+      <c r="J187" s="4"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B188" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C188" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D188" s="8">
+        <v>1.44</v>
+      </c>
+      <c r="E188" s="4"/>
+      <c r="F188" s="4"/>
+      <c r="G188" s="4"/>
+      <c r="H188" s="4"/>
+      <c r="I188" s="4"/>
+      <c r="J188" s="4"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B189" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C189" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D189" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E189" s="4"/>
+      <c r="F189" s="4"/>
+      <c r="G189" s="4"/>
+      <c r="H189" s="4"/>
+      <c r="I189" s="4"/>
+      <c r="J189" s="4"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B190" s="6">
+        <v>0.61</v>
+      </c>
+      <c r="C190" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D190" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E190" s="4"/>
+      <c r="F190" s="4"/>
+      <c r="G190" s="4"/>
+      <c r="H190" s="4"/>
+      <c r="I190" s="4"/>
+      <c r="J190" s="4"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B191" s="6">
+        <v>0.82</v>
+      </c>
+      <c r="C191" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D191" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="E191" s="4"/>
+      <c r="F191" s="4"/>
+      <c r="G191" s="4"/>
+      <c r="H191" s="4"/>
+      <c r="I191" s="4"/>
+      <c r="J191" s="4"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="B192" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="C192" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D192" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E192" s="4"/>
+      <c r="F192" s="4"/>
+      <c r="G192" s="4"/>
+      <c r="H192" s="4"/>
+      <c r="I192" s="4"/>
+      <c r="J192" s="4"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B193" s="6">
+        <v>0.68</v>
+      </c>
+      <c r="C193" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D193" s="8">
+        <v>3.25</v>
+      </c>
+      <c r="E193" s="4"/>
+      <c r="F193" s="4"/>
+      <c r="G193" s="4"/>
+      <c r="H193" s="4"/>
+      <c r="I193" s="4"/>
+      <c r="J193" s="4"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B194" s="6">
+        <v>0.88</v>
+      </c>
+      <c r="C194" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D194" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E194" s="4"/>
+      <c r="F194" s="4"/>
+      <c r="G194" s="4"/>
+      <c r="H194" s="4"/>
+      <c r="I194" s="4"/>
+      <c r="J194" s="4"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B195" s="6">
+        <v>0.72</v>
+      </c>
+      <c r="C195" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D195" s="8">
+        <v>1.33</v>
+      </c>
+      <c r="E195" s="4"/>
+      <c r="F195" s="4"/>
+      <c r="G195" s="4"/>
+      <c r="H195" s="4"/>
+      <c r="I195" s="4"/>
+      <c r="J195" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: super analizador con umbrales de acierto configurables por stake y fórmula con rangos exactos
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="35">
   <si>
     <t>Jugador / Favorito</t>
   </si>
@@ -37,6 +37,9 @@
     <t>SI</t>
   </si>
   <si>
+    <t>Cezar Cretu</t>
+  </si>
+  <si>
     <t>Denis Yevseyev</t>
   </si>
   <si>
@@ -55,7 +58,13 @@
     <t>Imanol Lopez Morillo</t>
   </si>
   <si>
+    <t>Inaki Montes De La Torre</t>
+  </si>
+  <si>
     <t>Juan Bautista Otegui</t>
+  </si>
+  <si>
+    <t>Juan Estevez</t>
   </si>
   <si>
     <t>Manas Dhamne</t>
@@ -493,13 +502,13 @@
         <v>8</v>
       </c>
       <c r="B4" s="6">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="8">
-        <v>1.72</v>
+        <v>1.61</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -510,13 +519,13 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="6">
-        <v>0.68</v>
+        <v>0.61</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="8">
         <v>1.72</v>
@@ -533,13 +542,13 @@
         <v>9</v>
       </c>
       <c r="B6" s="6">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D6" s="8">
-        <v>1.9</v>
+        <v>1.72</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
@@ -550,10 +559,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="6">
-        <v>0.66</v>
+        <v>0.63</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>7</v>
@@ -573,13 +582,13 @@
         <v>10</v>
       </c>
       <c r="B8" s="6">
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="8">
-        <v>1.61</v>
+        <v>1.9</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
@@ -593,13 +602,13 @@
         <v>11</v>
       </c>
       <c r="B9" s="6">
-        <v>0.85</v>
+        <v>0.64</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="8">
-        <v>1.5</v>
+        <v>1.61</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
@@ -613,13 +622,13 @@
         <v>12</v>
       </c>
       <c r="B10" s="6">
-        <v>0.72</v>
+        <v>0.85</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="8">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -633,13 +642,13 @@
         <v>13</v>
       </c>
       <c r="B11" s="6">
-        <v>0.67</v>
+        <v>0.72</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="8">
-        <v>1.83</v>
+        <v>2.1</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
@@ -653,10 +662,10 @@
         <v>14</v>
       </c>
       <c r="B12" s="6">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" s="8">
         <v>1.83</v>
@@ -673,10 +682,10 @@
         <v>15</v>
       </c>
       <c r="B13" s="6">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="8">
         <v>1.53</v>
@@ -693,13 +702,13 @@
         <v>16</v>
       </c>
       <c r="B14" s="6">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="8">
-        <v>1.53</v>
+        <v>1.83</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -713,13 +722,13 @@
         <v>17</v>
       </c>
       <c r="B15" s="6">
-        <v>0.56</v>
+        <v>0.63</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D15" s="8">
-        <v>1.66</v>
+        <v>1.61</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
@@ -730,16 +739,16 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" s="6">
-        <v>0.61</v>
+        <v>0.68</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D16" s="8">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -750,7 +759,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17" s="6">
         <v>0.62</v>
@@ -759,7 +768,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="8">
-        <v>2.1</v>
+        <v>1.53</v>
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
@@ -770,16 +779,16 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" s="6">
-        <v>0.64</v>
+        <v>0.56</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="8">
-        <v>1.44</v>
+        <v>1.66</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -793,13 +802,13 @@
         <v>20</v>
       </c>
       <c r="B19" s="6">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="8">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -813,13 +822,13 @@
         <v>20</v>
       </c>
       <c r="B20" s="6">
-        <v>0.82</v>
+        <v>0.75</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D20" s="8">
-        <v>1.5</v>
+        <v>2.37</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -833,13 +842,13 @@
         <v>21</v>
       </c>
       <c r="B21" s="6">
-        <v>0.57</v>
+        <v>0.62</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="8">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -853,13 +862,13 @@
         <v>22</v>
       </c>
       <c r="B22" s="6">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="8">
-        <v>2.0</v>
+        <v>1.44</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -873,13 +882,13 @@
         <v>23</v>
       </c>
       <c r="B23" s="6">
-        <v>0.64</v>
+        <v>0.72</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D23" s="8">
-        <v>1.53</v>
+        <v>2.5</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
@@ -890,16 +899,16 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="6">
-        <v>0.64</v>
+        <v>0.82</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="8">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -919,7 +928,7 @@
         <v>7</v>
       </c>
       <c r="D25" s="8">
-        <v>1.61</v>
+        <v>1.4</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
@@ -933,13 +942,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="6">
-        <v>0.58</v>
+        <v>0.62</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="8">
-        <v>1.72</v>
+        <v>2.0</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -953,13 +962,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="6">
-        <v>0.68</v>
+        <v>0.64</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D27" s="8">
-        <v>1.66</v>
+        <v>1.53</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -970,16 +979,16 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" s="6">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="8">
-        <v>1.4</v>
+        <v>1.61</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
@@ -993,13 +1002,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="6">
-        <v>0.78</v>
+        <v>0.57</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D29" s="8">
-        <v>1.66</v>
+        <v>1.61</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
@@ -1010,16 +1019,16 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" s="6">
-        <v>0.58</v>
+        <v>0.56</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D30" s="8">
-        <v>2.0</v>
+        <v>1.8</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
@@ -1030,16 +1039,16 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" s="6">
-        <v>0.71</v>
+        <v>0.58</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="8">
-        <v>1.83</v>
+        <v>1.72</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
@@ -1053,13 +1062,13 @@
         <v>29</v>
       </c>
       <c r="B32" s="6">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="8">
-        <v>1.61</v>
+        <v>1.66</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
@@ -1070,16 +1079,16 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" s="6">
-        <v>0.71</v>
+        <v>0.65</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D33" s="8">
-        <v>1.61</v>
+        <v>1.4</v>
       </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
@@ -1090,16 +1099,16 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B34" s="6">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="8">
-        <v>1.83</v>
+        <v>2.37</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
@@ -1109,6 +1118,18 @@
       <c r="J34" s="4"/>
     </row>
     <row r="35">
+      <c r="A35" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="8">
+        <v>1.66</v>
+      </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -1117,6 +1138,18 @@
       <c r="J35" s="4"/>
     </row>
     <row r="36">
+      <c r="A36" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B36" s="6">
+        <v>0.58</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="8">
+        <v>2.0</v>
+      </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -1125,6 +1158,18 @@
       <c r="J36" s="4"/>
     </row>
     <row r="37">
+      <c r="A37" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="8">
+        <v>1.83</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -1133,6 +1178,18 @@
       <c r="J37" s="4"/>
     </row>
     <row r="38">
+      <c r="A38" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="6">
+        <v>0.64</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="8">
+        <v>1.61</v>
+      </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -1141,6 +1198,18 @@
       <c r="J38" s="4"/>
     </row>
     <row r="39">
+      <c r="A39" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="6">
+        <v>0.63</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="8">
+        <v>1.57</v>
+      </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -1149,6 +1218,18 @@
       <c r="J39" s="4"/>
     </row>
     <row r="40">
+      <c r="A40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="8">
+        <v>1.61</v>
+      </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -1157,6 +1238,18 @@
       <c r="J40" s="4"/>
     </row>
     <row r="41">
+      <c r="A41" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="6">
+        <v>0.62</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="8">
+        <v>1.83</v>
+      </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -2332,41 +2425,9 @@
       <c r="I187" s="4"/>
       <c r="J187" s="4"/>
     </row>
-    <row r="188">
-      <c r="E188" s="4"/>
-      <c r="F188" s="4"/>
-      <c r="G188" s="4"/>
-      <c r="H188" s="4"/>
-      <c r="I188" s="4"/>
-      <c r="J188" s="4"/>
-    </row>
-    <row r="189">
-      <c r="E189" s="4"/>
-      <c r="F189" s="4"/>
-      <c r="G189" s="4"/>
-      <c r="H189" s="4"/>
-      <c r="I189" s="4"/>
-      <c r="J189" s="4"/>
-    </row>
-    <row r="190">
-      <c r="E190" s="4"/>
-      <c r="F190" s="4"/>
-      <c r="G190" s="4"/>
-      <c r="H190" s="4"/>
-      <c r="I190" s="4"/>
-      <c r="J190" s="4"/>
-    </row>
-    <row r="191">
-      <c r="E191" s="4"/>
-      <c r="F191" s="4"/>
-      <c r="G191" s="4"/>
-      <c r="H191" s="4"/>
-      <c r="I191" s="4"/>
-      <c r="J191" s="4"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C34">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C41">
       <formula1>"NO,SI"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>